<commit_message>
Update osworld_verified_results.xlsx with new verified data
</commit_message>
<xml_diff>
--- a/static/data/osworld_verified_results.xlsx
+++ b/static/data/osworld_verified_results.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="13260"/>
+    <workbookView windowWidth="27660" windowHeight="13280"/>
   </bookViews>
   <sheets>
     <sheet name="Eval Results" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2518" uniqueCount="778">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2537" uniqueCount="792">
   <si>
     <t>Model</t>
   </si>
@@ -2361,6 +2361,48 @@
   </si>
   <si>
     <t>13.84/17</t>
+  </si>
+  <si>
+    <t>GUI-Owl-1.5 32B</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/abs/2602.16855</t>
+  </si>
+  <si>
+    <t>Mobile-Agent Team</t>
+  </si>
+  <si>
+    <t>197.37/356</t>
+  </si>
+  <si>
+    <t>29.96/45</t>
+  </si>
+  <si>
+    <t>20.0/26</t>
+  </si>
+  <si>
+    <t>23.0/47</t>
+  </si>
+  <si>
+    <t>29.99/47</t>
+  </si>
+  <si>
+    <t>14.0/23</t>
+  </si>
+  <si>
+    <t>25.43/93</t>
+  </si>
+  <si>
+    <t>16.0/21</t>
+  </si>
+  <si>
+    <t>13.0/15</t>
+  </si>
+  <si>
+    <t>5.99/16</t>
+  </si>
+  <si>
+    <t>20.0/23</t>
   </si>
 </sst>
 </file>
@@ -13602,29 +13644,73 @@
       <c r="AB135" s="4"/>
       <c r="AC135" s="4"/>
     </row>
-    <row r="136" ht="15.15" spans="1:29">
-      <c r="A136" s="4"/>
-      <c r="B136" s="4"/>
-      <c r="C136" s="4"/>
-      <c r="D136" s="4"/>
-      <c r="E136" s="4"/>
-      <c r="F136" s="4"/>
-      <c r="G136" s="4"/>
-      <c r="H136" s="4"/>
-      <c r="I136" s="4"/>
-      <c r="J136" s="4"/>
-      <c r="K136" s="4"/>
-      <c r="L136" s="4"/>
-      <c r="M136" s="4"/>
-      <c r="N136" s="4"/>
-      <c r="O136" s="4"/>
-      <c r="P136" s="4"/>
-      <c r="Q136" s="4"/>
-      <c r="R136" s="4"/>
-      <c r="S136" s="4"/>
-      <c r="T136" s="4"/>
-      <c r="U136" s="4"/>
-      <c r="V136" s="4"/>
+    <row r="136" ht="29.75" spans="1:29">
+      <c r="A136" s="3" t="s">
+        <v>778</v>
+      </c>
+      <c r="B136" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>779</v>
+      </c>
+      <c r="D136" s="3" t="s">
+        <v>780</v>
+      </c>
+      <c r="E136" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F136" s="7">
+        <v>50</v>
+      </c>
+      <c r="G136" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H136" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I136" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J136" s="14">
+        <v>46108</v>
+      </c>
+      <c r="K136" s="7">
+        <v>55.44</v>
+      </c>
+      <c r="L136" s="3" t="s">
+        <v>781</v>
+      </c>
+      <c r="M136" s="3" t="s">
+        <v>782</v>
+      </c>
+      <c r="N136" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="O136" s="3" t="s">
+        <v>784</v>
+      </c>
+      <c r="P136" s="3" t="s">
+        <v>785</v>
+      </c>
+      <c r="Q136" s="3" t="s">
+        <v>786</v>
+      </c>
+      <c r="R136" s="3" t="s">
+        <v>787</v>
+      </c>
+      <c r="S136" s="3" t="s">
+        <v>788</v>
+      </c>
+      <c r="T136" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="U136" s="3" t="s">
+        <v>790</v>
+      </c>
+      <c r="V136" s="3" t="s">
+        <v>791</v>
+      </c>
       <c r="W136" s="4"/>
       <c r="X136" s="4"/>
       <c r="Y136" s="4"/>
@@ -42932,6 +43018,7 @@
     <hyperlink ref="C133" r:id="rId37" display="https://github.com/MoonshotAI/Kimi-K2.5/blob/master/tech_report.pdf" tooltip="https://github.com/MoonshotAI/Kimi-K2.5/blob/master/tech_report.pdf"/>
     <hyperlink ref="C134" r:id="rId38" display="https://github.com/wadang/muscle-mem-agent" tooltip="https://github.com/wadang/muscle-mem-agent"/>
     <hyperlink ref="C135" r:id="rId39" display="https://www.anthropic.com/news/claude-sonnet-4-6" tooltip="https://www.anthropic.com/news/claude-sonnet-4-6"/>
+    <hyperlink ref="C136" r:id="rId40" display="https://arxiv.org/abs/2602.16855" tooltip="https://arxiv.org/abs/2602.16855"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update osworld_verified_results.xlsx with latest verified data revisions
</commit_message>
<xml_diff>
--- a/static/data/osworld_verified_results.xlsx
+++ b/static/data/osworld_verified_results.xlsx
@@ -12307,8 +12307,8 @@
       <c r="D118" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E118" s="10" t="s">
-        <v>74</v>
+      <c r="E118" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="F118" s="7">
         <v>100</v>

</xml_diff>

<commit_message>
Update osworld_verified_results.xlsx with new verified results
</commit_message>
<xml_diff>
--- a/static/data/osworld_verified_results.xlsx
+++ b/static/data/osworld_verified_results.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="13320"/>
+    <workbookView windowWidth="27660" windowHeight="13280"/>
   </bookViews>
   <sheets>
     <sheet name="Eval Results" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2688" uniqueCount="867">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2707" uniqueCount="878">
   <si>
     <t>Model</t>
   </si>
@@ -2628,6 +2628,39 @@
   </si>
   <si>
     <t>14.0/17</t>
+  </si>
+  <si>
+    <t>MiniMax M3</t>
+  </si>
+  <si>
+    <t>MiniMax</t>
+  </si>
+  <si>
+    <t>https://www.minimaxi.com/blog/minimax-m3</t>
+  </si>
+  <si>
+    <t>MiniMax Team</t>
+  </si>
+  <si>
+    <t>269.18 / 358</t>
+  </si>
+  <si>
+    <t>34.96/46</t>
+  </si>
+  <si>
+    <t>38.0/47</t>
+  </si>
+  <si>
+    <t>34.63/47</t>
+  </si>
+  <si>
+    <t>20.97/23</t>
+  </si>
+  <si>
+    <t>56.64/92</t>
+  </si>
+  <si>
+    <t>12.99/15</t>
   </si>
 </sst>
 </file>
@@ -14547,29 +14580,73 @@
       <c r="AB144" s="4"/>
       <c r="AC144" s="4"/>
     </row>
-    <row r="145" ht="15.15" spans="1:29">
-      <c r="A145" s="4"/>
-      <c r="B145" s="4"/>
-      <c r="C145" s="4"/>
-      <c r="D145" s="4"/>
-      <c r="E145" s="4"/>
-      <c r="F145" s="4"/>
-      <c r="G145" s="4"/>
-      <c r="H145" s="4"/>
-      <c r="I145" s="4"/>
-      <c r="J145" s="4"/>
-      <c r="K145" s="4"/>
-      <c r="L145" s="4"/>
-      <c r="M145" s="4"/>
-      <c r="N145" s="4"/>
-      <c r="O145" s="4"/>
-      <c r="P145" s="4"/>
-      <c r="Q145" s="4"/>
-      <c r="R145" s="4"/>
-      <c r="S145" s="4"/>
-      <c r="T145" s="4"/>
-      <c r="U145" s="4"/>
-      <c r="V145" s="4"/>
+    <row r="145" spans="1:29">
+      <c r="A145" s="3" t="s">
+        <v>867</v>
+      </c>
+      <c r="B145" s="3" t="s">
+        <v>868</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>869</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>870</v>
+      </c>
+      <c r="E145" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F145" s="7">
+        <v>100</v>
+      </c>
+      <c r="G145" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H145" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="I145" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J145" s="14">
+        <v>46181</v>
+      </c>
+      <c r="K145" s="7">
+        <v>75.19</v>
+      </c>
+      <c r="L145" s="3" t="s">
+        <v>871</v>
+      </c>
+      <c r="M145" s="3" t="s">
+        <v>872</v>
+      </c>
+      <c r="N145" s="3" t="s">
+        <v>783</v>
+      </c>
+      <c r="O145" s="3" t="s">
+        <v>873</v>
+      </c>
+      <c r="P145" s="3" t="s">
+        <v>874</v>
+      </c>
+      <c r="Q145" s="3" t="s">
+        <v>875</v>
+      </c>
+      <c r="R145" s="3" t="s">
+        <v>876</v>
+      </c>
+      <c r="S145" s="3" t="s">
+        <v>811</v>
+      </c>
+      <c r="T145" s="3" t="s">
+        <v>789</v>
+      </c>
+      <c r="U145" s="3" t="s">
+        <v>877</v>
+      </c>
+      <c r="V145" s="3" t="s">
+        <v>699</v>
+      </c>
       <c r="W145" s="4"/>
       <c r="X145" s="4"/>
       <c r="Y145" s="4"/>
@@ -43607,6 +43684,7 @@
     <hyperlink ref="C142" r:id="rId45" display="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota" tooltip="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota"/>
     <hyperlink ref="C143" r:id="rId45" display="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota" tooltip="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota"/>
     <hyperlink ref="C144" r:id="rId46" display="https://qwen.ai/blog?id=qwen3.7" tooltip="https://qwen.ai/blog?id=qwen3.7"/>
+    <hyperlink ref="C145" r:id="rId47" display="https://www.minimaxi.com/blog/minimax-m3" tooltip="https://www.minimaxi.com/blog/minimax-m3"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
Update verified results data
</commit_message>
<xml_diff>
--- a/static/data/osworld_verified_results.xlsx
+++ b/static/data/osworld_verified_results.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="27660" windowHeight="13280"/>
+    <workbookView windowWidth="27660" windowHeight="13320"/>
   </bookViews>
   <sheets>
     <sheet name="Eval Results" sheetId="2" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2707" uniqueCount="878">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2726" uniqueCount="887">
   <si>
     <t>Model</t>
   </si>
@@ -2661,6 +2661,33 @@
   </si>
   <si>
     <t>12.99/15</t>
+  </si>
+  <si>
+    <t>Coasty CUA v1</t>
+  </si>
+  <si>
+    <t>Coasty Team</t>
+  </si>
+  <si>
+    <t>https://coasty.ai</t>
+  </si>
+  <si>
+    <t>297.29 / 359</t>
+  </si>
+  <si>
+    <t>25.00/26</t>
+  </si>
+  <si>
+    <t>44.96/47</t>
+  </si>
+  <si>
+    <t>64.39/93</t>
+  </si>
+  <si>
+    <t>24.00/24</t>
+  </si>
+  <si>
+    <t>11.99/15</t>
   </si>
 </sst>
 </file>
@@ -14655,29 +14682,73 @@
       <c r="AB145" s="4"/>
       <c r="AC145" s="4"/>
     </row>
-    <row r="146" ht="15.15" spans="1:29">
-      <c r="A146" s="4"/>
-      <c r="B146" s="4"/>
-      <c r="C146" s="4"/>
-      <c r="D146" s="4"/>
-      <c r="E146" s="4"/>
-      <c r="F146" s="4"/>
-      <c r="G146" s="4"/>
-      <c r="H146" s="4"/>
-      <c r="I146" s="4"/>
-      <c r="J146" s="4"/>
-      <c r="K146" s="4"/>
-      <c r="L146" s="4"/>
-      <c r="M146" s="4"/>
-      <c r="N146" s="4"/>
-      <c r="O146" s="4"/>
-      <c r="P146" s="4"/>
-      <c r="Q146" s="4"/>
-      <c r="R146" s="4"/>
-      <c r="S146" s="4"/>
-      <c r="T146" s="4"/>
-      <c r="U146" s="4"/>
-      <c r="V146" s="4"/>
+    <row r="146" spans="1:29">
+      <c r="A146" s="15" t="s">
+        <v>878</v>
+      </c>
+      <c r="B146" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>880</v>
+      </c>
+      <c r="D146" s="3" t="s">
+        <v>879</v>
+      </c>
+      <c r="E146" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="F146" s="7">
+        <v>100</v>
+      </c>
+      <c r="G146" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H146" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="I146" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="J146" s="14">
+        <v>46204</v>
+      </c>
+      <c r="K146" s="7">
+        <v>82.81</v>
+      </c>
+      <c r="L146" s="3" t="s">
+        <v>881</v>
+      </c>
+      <c r="M146" s="15" t="s">
+        <v>618</v>
+      </c>
+      <c r="N146" s="15" t="s">
+        <v>882</v>
+      </c>
+      <c r="O146" s="15" t="s">
+        <v>833</v>
+      </c>
+      <c r="P146" s="15" t="s">
+        <v>883</v>
+      </c>
+      <c r="Q146" s="15" t="s">
+        <v>452</v>
+      </c>
+      <c r="R146" s="15" t="s">
+        <v>884</v>
+      </c>
+      <c r="S146" s="15" t="s">
+        <v>885</v>
+      </c>
+      <c r="T146" s="15" t="s">
+        <v>821</v>
+      </c>
+      <c r="U146" s="15" t="s">
+        <v>886</v>
+      </c>
+      <c r="V146" s="15" t="s">
+        <v>823</v>
+      </c>
       <c r="W146" s="4"/>
       <c r="X146" s="4"/>
       <c r="Y146" s="4"/>
@@ -43685,6 +43756,7 @@
     <hyperlink ref="C143" r:id="rId45" display="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota" tooltip="https://pointer.ai/blog/sota?utm_source=osworld&amp;utm_medium=leaderboard&amp;utm_campaign=sota"/>
     <hyperlink ref="C144" r:id="rId46" display="https://qwen.ai/blog?id=qwen3.7" tooltip="https://qwen.ai/blog?id=qwen3.7"/>
     <hyperlink ref="C145" r:id="rId47" display="https://www.minimaxi.com/blog/minimax-m3" tooltip="https://www.minimaxi.com/blog/minimax-m3"/>
+    <hyperlink ref="C146" r:id="rId48" display="https://coasty.ai" tooltip="https://coasty.ai"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>